<commit_message>
Figure and content generation for Chapter 3
</commit_message>
<xml_diff>
--- a/Chapter3/Tables/Reduced01_112123SalAspIrr.xlsx
+++ b/Chapter3/Tables/Reduced01_112123SalAspIrr.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\Dissertation\Chapter3\Tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\DissertationBJT\Chapter3\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4C69F3-5472-4E08-ABEE-556D15DAC94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218D7F35-2CA8-4441-8AAA-8D08BBBA7A50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43095" yWindow="-2925" windowWidth="14610" windowHeight="15585" xr2:uid="{CCC1AB7D-2C6E-402E-ADA8-CFA773985701}"/>
+    <workbookView xWindow="28680" yWindow="-3045" windowWidth="29040" windowHeight="15720" xr2:uid="{CCC1AB7D-2C6E-402E-ADA8-CFA773985701}"/>
   </bookViews>
   <sheets>
     <sheet name="Reduced112123SalAspIrr" sheetId="1" r:id="rId1"/>
@@ -28555,7 +28555,7 @@
         <v>1.3571265158242658E-8</v>
       </c>
       <c r="M132" s="17">
-        <f t="shared" ref="M132:M163" si="73">(G132&lt;0.05)*J132+((G132&gt;=0.05)*(G132&lt;0.9))*K132+(G132&gt;=0.9)*L132</f>
+        <f t="shared" ref="M132:M140" si="73">(G132&lt;0.05)*J132+((G132&gt;=0.05)*(G132&lt;0.9))*K132+(G132&gt;=0.9)*L132</f>
         <v>8.0415456414707611E-10</v>
       </c>
       <c r="N132">
@@ -28579,7 +28579,7 @@
         <v>1.1599937331930819E-8</v>
       </c>
       <c r="T132">
-        <f t="shared" ref="T132:T163" si="78">(G132&lt;0.05)*Q132+((G132&gt;=0.05)*(G132&lt;0.9))*R132+(G132&gt;=0.9)*S132</f>
+        <f t="shared" ref="T132:T140" si="78">(G132&lt;0.05)*Q132+((G132&gt;=0.05)*(G132&lt;0.9))*R132+(G132&gt;=0.9)*S132</f>
         <v>6.8797188401058308E-10</v>
       </c>
       <c r="U132">

</xml_diff>